<commit_message>
media access via links
</commit_message>
<xml_diff>
--- a/student_management/static/student_management/downloads/sample_question_import.xlsx
+++ b/student_management/static/student_management/downloads/sample_question_import.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +28,25 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00111827"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,17 +54,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,16 +445,16 @@
   <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
@@ -444,88 +464,88 @@
     <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Option A</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Option B</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Option C</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Option D</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Option E</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Correct Answer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Explanation</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Has Question Image</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Has Option A Image</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Has Option B Image</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Has Option C Image</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Has Option D Image</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Has Option E Image</t>
         </is>

</xml_diff>